<commit_message>
Updated files for two scenarios
</commit_message>
<xml_diff>
--- a/Variability_table.xlsx
+++ b/Variability_table.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kajon\Documents\Spring 2026\RiverBasinManagement\Semester Project\773626e9b84248bc8d431da795ee1a16\data\contents\2_Drought_Hydrology_Scenarios\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kajon\Documents\GitHub\CEE6490_Spring2026_HydrologyBaseCase\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{29BDED9B-15DB-4EC7-97FF-9F7C4CCF00B0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{450E2410-C2DF-4E0C-9A18-003BCC5FD3CD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{743057FD-46D7-4E21-910F-BE3BBFC09D9D}"/>
   </bookViews>
@@ -2403,25 +2403,25 @@
       <sheetName val="RCP85_100"/>
     </sheetNames>
     <sheetDataSet>
-      <sheetData sheetId="0"/>
-      <sheetData sheetId="1"/>
-      <sheetData sheetId="2"/>
-      <sheetData sheetId="3"/>
-      <sheetData sheetId="4"/>
-      <sheetData sheetId="5"/>
-      <sheetData sheetId="6"/>
-      <sheetData sheetId="7"/>
-      <sheetData sheetId="8"/>
-      <sheetData sheetId="9"/>
-      <sheetData sheetId="10"/>
-      <sheetData sheetId="11"/>
-      <sheetData sheetId="12"/>
-      <sheetData sheetId="13"/>
-      <sheetData sheetId="14"/>
-      <sheetData sheetId="15"/>
-      <sheetData sheetId="16"/>
-      <sheetData sheetId="17"/>
-      <sheetData sheetId="18"/>
+      <sheetData sheetId="0" refreshError="1"/>
+      <sheetData sheetId="1" refreshError="1"/>
+      <sheetData sheetId="2" refreshError="1"/>
+      <sheetData sheetId="3" refreshError="1"/>
+      <sheetData sheetId="4" refreshError="1"/>
+      <sheetData sheetId="5" refreshError="1"/>
+      <sheetData sheetId="6" refreshError="1"/>
+      <sheetData sheetId="7" refreshError="1"/>
+      <sheetData sheetId="8" refreshError="1"/>
+      <sheetData sheetId="9" refreshError="1"/>
+      <sheetData sheetId="10" refreshError="1"/>
+      <sheetData sheetId="11" refreshError="1"/>
+      <sheetData sheetId="12" refreshError="1"/>
+      <sheetData sheetId="13" refreshError="1"/>
+      <sheetData sheetId="14" refreshError="1"/>
+      <sheetData sheetId="15" refreshError="1"/>
+      <sheetData sheetId="16" refreshError="1"/>
+      <sheetData sheetId="17" refreshError="1"/>
+      <sheetData sheetId="18" refreshError="1"/>
       <sheetData sheetId="19">
         <row r="2">
           <cell r="AU2">
@@ -2624,7 +2624,7 @@
           </cell>
         </row>
       </sheetData>
-      <sheetData sheetId="20"/>
+      <sheetData sheetId="20" refreshError="1"/>
       <sheetData sheetId="21">
         <row r="2">
           <cell r="AN2">
@@ -2827,13 +2827,13 @@
           </cell>
         </row>
       </sheetData>
-      <sheetData sheetId="22"/>
-      <sheetData sheetId="23"/>
-      <sheetData sheetId="24"/>
-      <sheetData sheetId="25"/>
-      <sheetData sheetId="26"/>
-      <sheetData sheetId="27"/>
-      <sheetData sheetId="28"/>
+      <sheetData sheetId="22" refreshError="1"/>
+      <sheetData sheetId="23" refreshError="1"/>
+      <sheetData sheetId="24" refreshError="1"/>
+      <sheetData sheetId="25" refreshError="1"/>
+      <sheetData sheetId="26" refreshError="1"/>
+      <sheetData sheetId="27" refreshError="1"/>
+      <sheetData sheetId="28" refreshError="1"/>
     </sheetDataSet>
   </externalBook>
 </externalLink>
@@ -3156,327 +3156,447 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C19080DC-D564-45B6-BDFC-9469BE84799D}">
-  <dimension ref="A1:B40"/>
+  <dimension ref="A1:C40"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1">
         <v>1</v>
       </c>
       <c r="B1">
         <v>0.54831462548262555</v>
       </c>
-    </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="C1">
+        <v>0.73501756696767417</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2">
         <v>2</v>
       </c>
       <c r="B2">
         <v>0.62325874903474909</v>
       </c>
-    </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="C2">
+        <v>0.83261321216375295</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3">
         <v>3</v>
       </c>
       <c r="B3">
         <v>1.173012972972973</v>
       </c>
-    </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="C3">
+        <v>0.95457148396566027</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4">
         <v>4</v>
       </c>
       <c r="B4">
         <v>0.75279770656370659</v>
       </c>
-    </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="C4">
+        <v>1.359376390210278</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5">
         <v>5</v>
       </c>
       <c r="B5">
         <v>0.54831462548262555</v>
       </c>
-    </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="C5">
+        <v>1.4456991373049499</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6">
         <v>6</v>
       </c>
       <c r="B6">
         <v>0.97237374517374531</v>
       </c>
-    </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="C6">
+        <v>1.1312229009476988</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A7">
         <v>7</v>
       </c>
       <c r="B7">
         <v>0.62210343629343634</v>
       </c>
-    </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="C7">
+        <v>1.2264756399374519</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A8">
         <v>8</v>
       </c>
       <c r="B8">
         <v>1.3240520463320464</v>
       </c>
-    </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="C8">
+        <v>1.2755815308975986</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A9">
         <v>9</v>
       </c>
       <c r="B9">
         <v>0.43326071814671813</v>
       </c>
-    </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="C9">
+        <v>0.80824415313826259</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A10">
         <v>10</v>
       </c>
       <c r="B10">
         <v>1.4245233204633205</v>
       </c>
-    </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="C10">
+        <v>1.0777455255113437</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A11">
         <v>11</v>
       </c>
       <c r="B11">
         <v>0.54831462548262555</v>
       </c>
-    </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="C11">
+        <v>1.4892336753565794</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A12">
         <v>12</v>
       </c>
       <c r="B12">
         <v>0.8065713513513515</v>
       </c>
-    </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="C12">
+        <v>1.0910590920195291</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A13">
         <v>13</v>
       </c>
       <c r="B13">
         <v>0.63131714285714291</v>
       </c>
-    </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="C13">
+        <v>0.91073826442451744</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A14">
         <v>14</v>
       </c>
       <c r="B14">
         <v>0.52311826254826255</v>
       </c>
-    </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="C14">
+        <v>0.94865633211014677</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A15">
         <v>15</v>
       </c>
       <c r="B15">
         <v>0.84902671814671826</v>
       </c>
-    </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="C15">
+        <v>0.58340480311432896</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A16">
         <v>16</v>
       </c>
       <c r="B16">
         <v>0.97237374517374531</v>
       </c>
-    </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="C16">
+        <v>0.84180985302657918</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A17">
         <v>17</v>
       </c>
       <c r="B17">
         <v>0.97237374517374531</v>
       </c>
-    </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="C17">
+        <v>1.6655583798844866</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A18">
         <v>18</v>
       </c>
       <c r="B18">
         <v>0.62210343629343634</v>
       </c>
-    </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="C18">
+        <v>1.1365009497941854</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A19">
         <v>19</v>
       </c>
       <c r="B19">
         <v>0.52311826254826255</v>
       </c>
-    </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="C19">
+        <v>1.4365315756597146</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A20">
         <v>20</v>
       </c>
       <c r="B20">
         <v>1.0181155984555985</v>
       </c>
-    </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="C20">
+        <v>1.0775961359839152</v>
+      </c>
+    </row>
+    <row r="21" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A21">
         <v>21</v>
       </c>
       <c r="B21">
         <v>0.64108096525096525</v>
       </c>
-    </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="C21">
+        <v>1.0650683861003862</v>
+      </c>
+    </row>
+    <row r="22" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A22">
         <v>22</v>
       </c>
       <c r="B22">
         <v>0.92772694980694981</v>
       </c>
-    </row>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="C22">
+        <v>1.1919540881840462</v>
+      </c>
+    </row>
+    <row r="23" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A23">
         <v>23</v>
       </c>
       <c r="B23">
         <v>0.64108096525096525</v>
       </c>
-    </row>
-    <row r="24" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="C23">
+        <v>1.0626419039280077</v>
+      </c>
+    </row>
+    <row r="24" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A24">
         <v>24</v>
       </c>
       <c r="B24">
         <v>0.54831462548262555</v>
       </c>
-    </row>
-    <row r="25" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="C24">
+        <v>1.1239607666868727</v>
+      </c>
+    </row>
+    <row r="25" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A25">
         <v>25</v>
       </c>
       <c r="B25">
         <v>0.54831462548262555</v>
       </c>
-    </row>
-    <row r="26" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="C25">
+        <v>0.95003007376112747</v>
+      </c>
+    </row>
+    <row r="26" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A26">
         <v>26</v>
       </c>
       <c r="B26">
         <v>1.4245233204633205</v>
       </c>
-    </row>
-    <row r="27" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="C26">
+        <v>1.1894426901687953</v>
+      </c>
+    </row>
+    <row r="27" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A27">
         <v>27</v>
       </c>
       <c r="B27">
         <v>0.62325874903474909</v>
       </c>
-    </row>
-    <row r="28" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="C27">
+        <v>1.0695210277800773</v>
+      </c>
+    </row>
+    <row r="28" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A28">
         <v>28</v>
       </c>
       <c r="B28">
         <v>1.4245233204633205</v>
       </c>
-    </row>
-    <row r="29" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="C28">
+        <v>1.1437135321994905</v>
+      </c>
+    </row>
+    <row r="29" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A29">
         <v>29</v>
       </c>
       <c r="B29">
         <v>1.0181155984555985</v>
       </c>
-    </row>
-    <row r="30" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="C29">
+        <v>0.87062647175723551</v>
+      </c>
+    </row>
+    <row r="30" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A30">
         <v>30</v>
       </c>
       <c r="B30">
         <v>0.8065713513513515</v>
       </c>
-    </row>
-    <row r="31" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="C30">
+        <v>1.0949955443121933</v>
+      </c>
+    </row>
+    <row r="31" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A31">
         <v>31</v>
       </c>
       <c r="B31">
         <v>0.54831462548262555</v>
       </c>
-    </row>
-    <row r="32" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="C31">
+        <v>1.0532551171128572</v>
+      </c>
+    </row>
+    <row r="32" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A32">
         <v>32</v>
       </c>
       <c r="B32">
         <v>0.80380455598455602</v>
       </c>
-    </row>
-    <row r="33" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="C32">
+        <v>0.98712122990522788</v>
+      </c>
+    </row>
+    <row r="33" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A33">
         <v>33</v>
       </c>
       <c r="B33">
         <v>0.62210343629343634</v>
       </c>
-    </row>
-    <row r="34" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="C33">
+        <v>1.0265157684929267</v>
+      </c>
+    </row>
+    <row r="34" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A34">
         <v>34</v>
       </c>
       <c r="B34">
         <v>0.62210343629343634</v>
       </c>
-    </row>
-    <row r="35" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="C34">
+        <v>0.83505583090717372</v>
+      </c>
+    </row>
+    <row r="35" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A35">
         <v>35</v>
       </c>
       <c r="B35">
         <v>1.4245233204633205</v>
       </c>
-    </row>
-    <row r="36" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="C35">
+        <v>0.58269320935575297</v>
+      </c>
+    </row>
+    <row r="36" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A36">
         <v>36</v>
       </c>
       <c r="B36">
         <v>0.62210343629343634</v>
       </c>
-    </row>
-    <row r="37" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="C36">
+        <v>0.73802668465490118</v>
+      </c>
+    </row>
+    <row r="37" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A37">
         <v>37</v>
       </c>
       <c r="B37">
         <v>0.54831462548262555</v>
       </c>
-    </row>
-    <row r="38" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="C37">
+        <v>1.1013330177478533</v>
+      </c>
+    </row>
+    <row r="38" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A38">
         <v>38</v>
       </c>
       <c r="B38">
         <v>0.63131714285714291</v>
       </c>
-    </row>
-    <row r="39" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="C38">
+        <v>0.81191009995213137</v>
+      </c>
+    </row>
+    <row r="39" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A39">
         <v>39</v>
       </c>
       <c r="B39">
         <v>0.84902671814671826</v>
       </c>
-    </row>
-    <row r="40" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="C39">
+        <v>0.85988666099109667</v>
+      </c>
+    </row>
+    <row r="40" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A40">
         <v>40</v>
       </c>
       <c r="B40">
         <v>0.94114579150579147</v>
+      </c>
+      <c r="C40">
+        <v>1.3719302108682472</v>
       </c>
     </row>
   </sheetData>

</xml_diff>